<commit_message>
refactor(core): extract session orchestration service
</commit_message>
<xml_diff>
--- a/tests/apollo_actual_output.xlsx
+++ b/tests/apollo_actual_output.xlsx
@@ -536,7 +536,7 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>EC4</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1141,7 +1141,7 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>INCLUDE</t>
+          <t>EXCLUDE</t>
         </is>
       </c>
     </row>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>EC3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1788,12 +1788,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>EC3</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1862,12 +1862,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>EC3</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">

</xml_diff>